<commit_message>
Gráficos da Distribuição Institucional
</commit_message>
<xml_diff>
--- a/Docs/Graficos.xlsx
+++ b/Docs/Graficos.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO1\Downloads\Fluxo-da-Comunicacao-Cientifica-Lic-Comp\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FCD5092F-65B0-403A-9640-E7442DC44FC1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{375D204A-F3B4-4FFC-AE35-4EC34BED406D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7425" xr2:uid="{AEC90C7E-1C91-4932-8D29-358D17889A45}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7425" activeTab="1" xr2:uid="{AEC90C7E-1C91-4932-8D29-358D17889A45}"/>
   </bookViews>
   <sheets>
     <sheet name="Panorama da Produção Cientifica" sheetId="1" r:id="rId1"/>
+    <sheet name="Distribuição Institucional" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="48">
   <si>
     <t>Ano</t>
   </si>
@@ -122,12 +123,60 @@
   <si>
     <t>Feminino</t>
   </si>
+  <si>
+    <t>Região</t>
+  </si>
+  <si>
+    <t>Sudoeste</t>
+  </si>
+  <si>
+    <t>Nordeste</t>
+  </si>
+  <si>
+    <t>Sul</t>
+  </si>
+  <si>
+    <t>Centro-Oeste</t>
+  </si>
+  <si>
+    <t>Norte</t>
+  </si>
+  <si>
+    <t>Instituições</t>
+  </si>
+  <si>
+    <t>Cursos</t>
+  </si>
+  <si>
+    <t>Qtd</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modalidade </t>
+  </si>
+  <si>
+    <t>A Distância</t>
+  </si>
+  <si>
+    <t>Presencial</t>
+  </si>
+  <si>
+    <t>Categoria Administrativa</t>
+  </si>
+  <si>
+    <t>Estadual</t>
+  </si>
+  <si>
+    <t>Federal</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -137,6 +186,13 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -176,10 +232,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -195,9 +252,20 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Porcentagem" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1506,6 +1574,566 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="pt-BR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Distribuição Institucional'!$B$10</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Instituições</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4">
+                  <a:lumMod val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-3959-4902-A40A-F3FBC23356C0}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000002-3959-4902-A40A-F3FBC23356C0}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="1"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="1"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000001-3959-4902-A40A-F3FBC23356C0}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="0"/>
+              <c:showCatName val="1"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="1"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000002-3959-4902-A40A-F3FBC23356C0}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:spPr>
+              <a:solidFill>
+                <a:sysClr val="window" lastClr="FFFFFF"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000">
+                    <a:lumMod val="25000"/>
+                    <a:lumOff val="75000"/>
+                  </a:sysClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="dk1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="pt-BR"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:spPr xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <a:prstGeom prst="wedgeRectCallout">
+                    <a:avLst/>
+                  </a:prstGeom>
+                  <a:noFill/>
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                </c15:spPr>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Distribuição Institucional'!$A$11:$A$12</c:f>
+              <c:strCache>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>A Distância</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Presencial</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Distribuição Institucional'!$B$11:$B$12</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>37</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-3959-4902-A40A-F3FBC23356C0}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="0"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="pt-BR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.78740157499999996" l="0.511811024" r="0.511811024" t="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="pt-BR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Distribuição Institucional'!$B$27</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Instituições</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6">
+                  <a:lumMod val="50000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000002-3B85-46C1-8532-F635C47E24C3}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2">
+                  <a:lumMod val="75000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-3B85-46C1-8532-F635C47E24C3}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dLbls>
+            <c:spPr>
+              <a:solidFill>
+                <a:sysClr val="window" lastClr="FFFFFF"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000">
+                    <a:lumMod val="25000"/>
+                    <a:lumOff val="75000"/>
+                  </a:sysClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="dk1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="pt-BR"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="1"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="1"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:spPr xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <a:prstGeom prst="wedgeRectCallout">
+                    <a:avLst/>
+                  </a:prstGeom>
+                  <a:noFill/>
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                </c15:spPr>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Distribuição Institucional'!$A$28:$A$29</c:f>
+              <c:strCache>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>Estadual</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Federal</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Distribuição Institucional'!$B$28:$B$29</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>26</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-3B85-46C1-8532-F635C47E24C3}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="0"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="pt-BR"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="pt-BR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.78740157499999996" l="0.511811024" r="0.511811024" t="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="12">
   <a:schemeClr val="accent2"/>
@@ -1623,6 +2251,86 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
   <cs:axisTitle>
@@ -2646,6 +3354,1044 @@
 </file>
 
 <file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -3269,6 +5015,83 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>257175</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>4762</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>600075</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>80962</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Gráfico 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{33408D6D-E99F-4028-A1BF-BCA83F43FC39}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>214312</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>176212</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>61912</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Gráfico 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C932AC20-8D45-4873-9AA8-67707CC2D974}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -3979,4 +5802,197 @@
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03EB4A3B-66C2-4F62-855F-FFB9D96FB5FC}">
+  <dimension ref="A1:E29"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="E1" s="8"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="7"/>
+      <c r="B2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" s="3">
+        <v>7</v>
+      </c>
+      <c r="C3" s="9">
+        <f>(B3/49)</f>
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="D3" s="2">
+        <v>6</v>
+      </c>
+      <c r="E3" s="10">
+        <f>(D3/33)</f>
+        <v>0.18181818181818182</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" s="3">
+        <v>21</v>
+      </c>
+      <c r="C4" s="9">
+        <f t="shared" ref="C4:C7" si="0">(B4/49)</f>
+        <v>0.42857142857142855</v>
+      </c>
+      <c r="D4" s="2">
+        <v>13</v>
+      </c>
+      <c r="E4" s="10">
+        <f t="shared" ref="E4:E7" si="1">(D4/33)</f>
+        <v>0.39393939393939392</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B5" s="3">
+        <v>8</v>
+      </c>
+      <c r="C5" s="9">
+        <f t="shared" si="0"/>
+        <v>0.16326530612244897</v>
+      </c>
+      <c r="D5" s="2">
+        <v>6</v>
+      </c>
+      <c r="E5" s="10">
+        <f t="shared" si="1"/>
+        <v>0.18181818181818182</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" s="3">
+        <v>4</v>
+      </c>
+      <c r="C6" s="9">
+        <f t="shared" si="0"/>
+        <v>8.1632653061224483E-2</v>
+      </c>
+      <c r="D6" s="2">
+        <v>4</v>
+      </c>
+      <c r="E6" s="10">
+        <f t="shared" si="1"/>
+        <v>0.12121212121212122</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B7" s="3">
+        <v>9</v>
+      </c>
+      <c r="C7" s="9">
+        <f t="shared" si="0"/>
+        <v>0.18367346938775511</v>
+      </c>
+      <c r="D7" s="2">
+        <v>4</v>
+      </c>
+      <c r="E7" s="10">
+        <f t="shared" si="1"/>
+        <v>0.12121212121212122</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" s="2">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B28" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B29" s="2">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="A1:A2"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>